<commit_message>
Update Project 1 monthly outputs
</commit_message>
<xml_diff>
--- a/Project_1_May2026_Update.xlsx
+++ b/Project_1_May2026_Update.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T17:26:51</t>
+          <t>2026-09-20T16:40:04</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
         <v>21.19</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>27.82298177528853</v>
+        <v>27.82296061656442</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>116</v>
@@ -839,13 +839,13 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0.02043076663695832</v>
+        <v>0.02043075292818304</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>27.46839945977315</v>
+        <v>27.46837891038678</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>6.278399459773151</v>
+        <v>6.278378910386781</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>3</v>
@@ -6955,7 +6955,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2.622556209564209</v>
+        <v>2.622556447982788</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -6963,10 +6963,10 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
-        <v>2.68250560760498</v>
+        <v>2.682507038116455</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0.0228591470497912</v>
+        <v>0.0228595995254095</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
@@ -6991,7 +6991,7 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>2.68250560760498</v>
+        <v>2.682507038116455</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -6999,10 +6999,10 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
-        <v>2.496466398239136</v>
+        <v>2.49646782875061</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-0.06935277556863939</v>
+        <v>-0.06935273858460167</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
@@ -7027,7 +7027,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2.496466398239136</v>
+        <v>2.49646782875061</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -7035,10 +7035,10 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2.67974066734314</v>
+        <v>2.679741382598877</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.07341347323291636</v>
+        <v>0.07341314465886306</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
@@ -7063,7 +7063,7 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>2.67974066734314</v>
+        <v>2.679741382598877</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         </is>
       </c>
       <c r="F5" s="3" t="n">
-        <v>2.565841436386108</v>
+        <v>2.565841197967529</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-0.04250382596535285</v>
+        <v>-0.04250417050352995</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
@@ -7099,7 +7099,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>2.565841436386108</v>
+        <v>2.565841197967529</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -7107,10 +7107,10 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>3.554834604263306</v>
+        <v>3.554834127426147</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.3854459413790421</v>
+        <v>0.3854458842745316</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -7135,7 +7135,7 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>3.554834604263306</v>
+        <v>3.554834127426147</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -7143,10 +7143,10 @@
         </is>
       </c>
       <c r="F7" s="3" t="n">
-        <v>3.560005664825439</v>
+        <v>3.56000542640686</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0.001454655740082078</v>
+        <v>0.001454723004039815</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -7171,7 +7171,7 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>3.560005664825439</v>
+        <v>3.56000542640686</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -7179,10 +7179,10 @@
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>4.002050399780273</v>
+        <v>4.002050876617432</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0.1241696717852019</v>
+        <v>0.1241698810152463</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -7207,7 +7207,7 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>4.002050399780273</v>
+        <v>4.002050876617432</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -7215,10 +7215,10 @@
         </is>
       </c>
       <c r="F9" s="3" t="n">
-        <v>4.176387310028076</v>
+        <v>4.176388263702393</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>0.04356189773556429</v>
+        <v>0.04356201169344254</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -7243,7 +7243,7 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>4.176387310028076</v>
+        <v>4.176388263702393</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -7254,7 +7254,7 @@
         <v>4.40635347366333</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0.05506341882685883</v>
+        <v>0.05506317790412329</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
@@ -7287,10 +7287,10 @@
         </is>
       </c>
       <c r="F11" s="3" t="n">
-        <v>5.097486972808838</v>
+        <v>5.097490310668945</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0.1568493093612204</v>
+        <v>0.1568500668719666</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -7315,7 +7315,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>5.097486972808838</v>
+        <v>5.097490310668945</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -7323,10 +7323,10 @@
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>4.95057201385498</v>
+        <v>4.950571060180664</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-0.02882105628470177</v>
+        <v>-0.02882187930417091</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -7351,7 +7351,7 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>4.95057201385498</v>
+        <v>4.950571060180664</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -7359,10 +7359,10 @@
         </is>
       </c>
       <c r="F13" s="3" t="n">
-        <v>4.772735595703125</v>
+        <v>4.772735118865967</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-0.03592239798838426</v>
+        <v>-0.03592230858882117</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
@@ -7387,7 +7387,7 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>4.772735595703125</v>
+        <v>4.772735118865967</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -7395,10 +7395,10 @@
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>6.062729358673096</v>
+        <v>6.062732696533203</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0.2702839361416431</v>
+        <v>0.2702847624139151</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
@@ -7423,7 +7423,7 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>6.062729358673096</v>
+        <v>6.062732696533203</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -7431,10 +7431,10 @@
         </is>
       </c>
       <c r="F15" s="3" t="n">
-        <v>5.972711563110352</v>
+        <v>5.97271203994751</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-0.01484773445048615</v>
+        <v>-0.01484819817920868</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -7459,7 +7459,7 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>5.972711563110352</v>
+        <v>5.97271203994751</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -7467,10 +7467,10 @@
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>5.715785980224609</v>
+        <v>5.715786457061768</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-0.04301657298715189</v>
+        <v>-0.04301656955288269</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -7495,7 +7495,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>5.715785980224609</v>
+        <v>5.715786457061768</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -7503,10 +7503,10 @@
         </is>
       </c>
       <c r="F17" s="3" t="n">
-        <v>5.550673484802246</v>
+        <v>5.550672054290771</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-0.02888710249012416</v>
+        <v>-0.02888743377860092</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -7531,7 +7531,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>5.550673484802246</v>
+        <v>5.550672054290771</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -7539,10 +7539,10 @@
         </is>
       </c>
       <c r="F18" s="3" t="n">
-        <v>6.228055953979492</v>
+        <v>6.228057384490967</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>0.1220360864374244</v>
+        <v>0.1220366333256104</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -7567,7 +7567,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>6.228055953979492</v>
+        <v>6.228057384490967</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -7575,10 +7575,10 @@
         </is>
       </c>
       <c r="F19" s="3" t="n">
-        <v>5.850456237792969</v>
+        <v>5.850456714630127</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>-0.06062882526693603</v>
+        <v>-0.06062896446669497</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -7603,7 +7603,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>5.850456237792969</v>
+        <v>5.850456714630127</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -7611,10 +7611,10 @@
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>6.047036647796631</v>
+        <v>6.047035217285156</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>0.03360086837908227</v>
+        <v>0.03360053962341936</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -7639,7 +7639,7 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>6.047036647796631</v>
+        <v>6.047035217285156</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
@@ -7647,10 +7647,10 @@
         </is>
       </c>
       <c r="F21" s="3" t="n">
-        <v>6.935433864593506</v>
+        <v>6.935433387756348</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0.1469144753935934</v>
+        <v>0.146914667857688</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
@@ -7675,7 +7675,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.935433864593506</v>
+        <v>6.935433387756348</v>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
@@ -7683,10 +7683,10 @@
         </is>
       </c>
       <c r="F22" s="3" t="n">
-        <v>6.943833827972412</v>
+        <v>6.943835258483887</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>0.001211166243223705</v>
+        <v>0.001211441341556485</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
@@ -7711,7 +7711,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>6.943833827972412</v>
+        <v>6.943835258483887</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
@@ -7719,10 +7719,10 @@
         </is>
       </c>
       <c r="F23" s="3" t="n">
-        <v>5.209483623504639</v>
+        <v>5.209482192993164</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>-0.2497683912712815</v>
+        <v>-0.249768751839513</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
@@ -7747,7 +7747,7 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>5.209483623504639</v>
+        <v>5.209482192993164</v>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
@@ -7755,10 +7755,10 @@
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>4.042298793792725</v>
+        <v>4.042298316955566</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-0.2240500045812026</v>
+        <v>-0.2240498830397153</v>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
@@ -7783,7 +7783,7 @@
         </is>
       </c>
       <c r="D25" s="3" t="n">
-        <v>4.042298793792725</v>
+        <v>4.042298316955566</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -7791,10 +7791,10 @@
         </is>
       </c>
       <c r="F25" s="3" t="n">
-        <v>3.302005052566528</v>
+        <v>3.302004814147949</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>-0.183136818674309</v>
+        <v>-0.1831367812965286</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
@@ -7819,7 +7819,7 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>3.302005052566528</v>
+        <v>3.302004814147949</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -7827,10 +7827,10 @@
         </is>
       </c>
       <c r="F26" s="3" t="n">
-        <v>3.555529832839966</v>
+        <v>3.555530071258545</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>0.07677904068510788</v>
+        <v>0.07677919063725391</v>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
@@ -7855,7 +7855,7 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>3.555529832839966</v>
+        <v>3.555530071258545</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
@@ -7863,10 +7863,10 @@
         </is>
       </c>
       <c r="F27" s="3" t="n">
-        <v>3.819417715072632</v>
+        <v>3.819417953491211</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>0.07421900381634172</v>
+        <v>0.07421899883953387</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -7891,7 +7891,7 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>3.819417715072632</v>
+        <v>3.819417953491211</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -7902,7 +7902,7 @@
         <v>4.445836544036865</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>0.1640089866296075</v>
+        <v>0.1640089139689633</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -7935,10 +7935,10 @@
         </is>
       </c>
       <c r="F29" s="3" t="n">
-        <v>4.481490135192871</v>
+        <v>4.481488704681396</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>0.008019546108555708</v>
+        <v>0.008019224344257836</v>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
@@ -7963,7 +7963,7 @@
         </is>
       </c>
       <c r="D30" s="3" t="n">
-        <v>4.481490135192871</v>
+        <v>4.481488704681396</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -7971,10 +7971,10 @@
         </is>
       </c>
       <c r="F30" s="3" t="n">
-        <v>3.357765674591064</v>
+        <v>3.357765436172485</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>-0.2507479491647804</v>
+        <v>-0.2507477632008893</v>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
@@ -7999,7 +7999,7 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>3.357765674591064</v>
+        <v>3.357765436172485</v>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
@@ -8007,10 +8007,10 @@
         </is>
       </c>
       <c r="F31" s="3" t="n">
-        <v>4.070911407470703</v>
+        <v>4.070912837982178</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>0.2123869864642927</v>
+        <v>0.212387498580785</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -8035,7 +8035,7 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>4.070911407470703</v>
+        <v>4.070912837982178</v>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
@@ -8046,7 +8046,7 @@
         <v>4.182209491729736</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>0.02733984435396586</v>
+        <v>0.02733948334858605</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -8079,10 +8079,10 @@
         </is>
       </c>
       <c r="F33" s="3" t="n">
-        <v>4.156326770782471</v>
+        <v>4.156326293945312</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>-0.006188767205097756</v>
+        <v>-0.006188881220705822</v>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
@@ -8107,7 +8107,7 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>4.156326770782471</v>
+        <v>4.156326293945312</v>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
@@ -8115,10 +8115,10 @@
         </is>
       </c>
       <c r="F34" s="3" t="n">
-        <v>4.319096088409424</v>
+        <v>4.319095134735107</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>0.03916181922248385</v>
+        <v>0.03916170898971694</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -8143,7 +8143,7 @@
         </is>
       </c>
       <c r="D35" s="3" t="n">
-        <v>4.319096088409424</v>
+        <v>4.319095134735107</v>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
@@ -8151,10 +8151,10 @@
         </is>
       </c>
       <c r="F35" s="3" t="n">
-        <v>4.987789630889893</v>
+        <v>4.987791061401367</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>0.154822566757649</v>
+        <v>0.1548231529536039</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -8179,7 +8179,7 @@
         </is>
       </c>
       <c r="D36" s="3" t="n">
-        <v>4.987789630889893</v>
+        <v>4.987791061401367</v>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
@@ -8187,10 +8187,10 @@
         </is>
       </c>
       <c r="F36" s="3" t="n">
-        <v>5.381809234619141</v>
+        <v>5.381811618804932</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>0.07899683685315129</v>
+        <v>0.07899700539838994</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -8215,7 +8215,7 @@
         </is>
       </c>
       <c r="D37" s="3" t="n">
-        <v>5.381809234619141</v>
+        <v>5.381811618804932</v>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
@@ -8223,10 +8223,10 @@
         </is>
       </c>
       <c r="F37" s="3" t="n">
-        <v>5.842668533325195</v>
+        <v>5.842667579650879</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>0.08563278232560179</v>
+        <v>0.08563212417834198</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -8251,7 +8251,7 @@
         </is>
       </c>
       <c r="D38" s="3" t="n">
-        <v>5.842668533325195</v>
+        <v>5.842667579650879</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
@@ -8262,7 +8262,7 @@
         <v>5.870727062225342</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>0.004802348231823794</v>
+        <v>0.004802512241529833</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -8295,10 +8295,10 @@
         </is>
       </c>
       <c r="F39" s="3" t="n">
-        <v>6.710042476654053</v>
+        <v>6.710043430328369</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>0.1429661787258361</v>
+        <v>0.1429663411715274</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -8323,7 +8323,7 @@
         </is>
       </c>
       <c r="D40" s="3" t="n">
-        <v>6.710042476654053</v>
+        <v>6.710043430328369</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
@@ -8331,10 +8331,10 @@
         </is>
       </c>
       <c r="F40" s="3" t="n">
-        <v>6.549293041229248</v>
+        <v>6.549293518066406</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>-0.02395654513128542</v>
+        <v>-0.0239566127896278</v>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>6.549293041229248</v>
+        <v>6.549293518066406</v>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
@@ -8370,7 +8370,7 @@
         <v>7.261864185333252</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>0.1088012308531945</v>
+        <v>0.1088011501242385</v>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
@@ -8439,10 +8439,10 @@
         </is>
       </c>
       <c r="F43" s="3" t="n">
-        <v>9.443387031555176</v>
+        <v>9.443389892578125</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.07059699667439601</v>
+        <v>0.07059732102863103</v>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
@@ -8467,7 +8467,7 @@
         </is>
       </c>
       <c r="D44" s="3" t="n">
-        <v>9.443387031555176</v>
+        <v>9.443389892578125</v>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
@@ -8478,7 +8478,7 @@
         <v>10.55399703979492</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>0.1176071683315141</v>
+        <v>0.1176068297349091</v>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
@@ -8619,10 +8619,10 @@
         </is>
       </c>
       <c r="F48" s="3" t="n">
-        <v>13.32878017425537</v>
+        <v>13.328782081604</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>0.06921160074748678</v>
+        <v>0.06921175375168209</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -8647,7 +8647,7 @@
         </is>
       </c>
       <c r="D49" s="3" t="n">
-        <v>13.32878017425537</v>
+        <v>13.328782081604</v>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
@@ -8655,10 +8655,10 @@
         </is>
       </c>
       <c r="F49" s="3" t="n">
-        <v>12.98799896240234</v>
+        <v>12.98799705505371</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>-0.02556732179522692</v>
+        <v>-0.02556760433653082</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -8683,7 +8683,7 @@
         </is>
       </c>
       <c r="D50" s="3" t="n">
-        <v>12.98799896240234</v>
+        <v>12.98799705505371</v>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
@@ -8694,7 +8694,7 @@
         <v>12.92308235168457</v>
       </c>
       <c r="G50" s="3" t="n">
-        <v>-0.004998199561433103</v>
+        <v>-0.004998053440725236</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
@@ -8727,10 +8727,10 @@
         </is>
       </c>
       <c r="F51" s="3" t="n">
-        <v>13.64411449432373</v>
+        <v>13.64411163330078</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>0.05579413045721027</v>
+        <v>0.05579390906862258</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
@@ -8755,7 +8755,7 @@
         </is>
       </c>
       <c r="D52" s="3" t="n">
-        <v>13.64411449432373</v>
+        <v>13.64411163330078</v>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
@@ -8763,10 +8763,10 @@
         </is>
       </c>
       <c r="F52" s="3" t="n">
-        <v>13.28432464599609</v>
+        <v>13.28432750701904</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>-0.02636960049531378</v>
+        <v>-0.02636918664632026</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
@@ -8791,7 +8791,7 @@
         </is>
       </c>
       <c r="D53" s="3" t="n">
-        <v>13.28432464599609</v>
+        <v>13.28432750701904</v>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
@@ -8799,10 +8799,10 @@
         </is>
       </c>
       <c r="F53" s="3" t="n">
-        <v>14.93761920928955</v>
+        <v>14.93762111663818</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>0.1244545437838092</v>
+        <v>0.1244544451908152</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
@@ -8827,7 +8827,7 @@
         </is>
       </c>
       <c r="D54" s="3" t="n">
-        <v>14.93761920928955</v>
+        <v>14.93762111663818</v>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
@@ -8838,7 +8838,7 @@
         <v>16.16670608520508</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>0.08228130993934912</v>
+        <v>0.08228117174547189</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
@@ -8907,10 +8907,10 @@
         </is>
       </c>
       <c r="F56" s="3" t="n">
-        <v>19.41006851196289</v>
+        <v>19.41006660461426</v>
       </c>
       <c r="G56" s="3" t="n">
-        <v>-0.02517175579831477</v>
+        <v>-0.02517185159072888</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
@@ -8935,7 +8935,7 @@
         </is>
       </c>
       <c r="D57" s="3" t="n">
-        <v>19.41006851196289</v>
+        <v>19.41006660461426</v>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
@@ -8943,10 +8943,10 @@
         </is>
       </c>
       <c r="F57" s="3" t="n">
-        <v>22.28683471679688</v>
+        <v>22.28683853149414</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>0.1482099974588429</v>
+        <v>0.1482103068206888</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
@@ -8971,7 +8971,7 @@
         </is>
       </c>
       <c r="D58" s="3" t="n">
-        <v>22.28683471679688</v>
+        <v>22.28683853149414</v>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
@@ -8979,10 +8979,10 @@
         </is>
       </c>
       <c r="F58" s="3" t="n">
-        <v>20.62515830993652</v>
+        <v>20.62515258789062</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>-0.07455865437939457</v>
+        <v>-0.07455906952685742</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
@@ -9007,7 +9007,7 @@
         </is>
       </c>
       <c r="D59" s="3" t="n">
-        <v>20.62515830993652</v>
+        <v>20.62515258789062</v>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
@@ -9015,10 +9015,10 @@
         </is>
       </c>
       <c r="F59" s="3" t="n">
-        <v>25.45487785339355</v>
+        <v>25.45488166809082</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>0.2341664229132356</v>
+        <v>0.2341669502622643</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
@@ -9043,7 +9043,7 @@
         </is>
       </c>
       <c r="D60" s="3" t="n">
-        <v>25.45487785339355</v>
+        <v>25.45488166809082</v>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
@@ -9051,10 +9051,10 @@
         </is>
       </c>
       <c r="F60" s="3" t="n">
-        <v>32.53269577026367</v>
+        <v>32.53270721435547</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>0.2780535014795418</v>
+        <v>0.2780537595323853</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
@@ -9079,7 +9079,7 @@
         </is>
       </c>
       <c r="D61" s="3" t="n">
-        <v>32.53269577026367</v>
+        <v>32.53270721435547</v>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
@@ -9090,7 +9090,7 @@
         <v>29.28561019897461</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>-0.09980991413127971</v>
+        <v>-0.09981023079284457</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
@@ -9123,10 +9123,10 @@
         </is>
       </c>
       <c r="F62" s="3" t="n">
-        <v>24.3816089630127</v>
+        <v>24.38160514831543</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>-0.1674542959030992</v>
+        <v>-0.1674544261615176</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
@@ -9151,7 +9151,7 @@
         </is>
       </c>
       <c r="D63" s="3" t="n">
-        <v>24.3816089630127</v>
+        <v>24.38160514831543</v>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
@@ -9159,10 +9159,10 @@
         </is>
       </c>
       <c r="F63" s="3" t="n">
-        <v>24.28103828430176</v>
+        <v>24.28104019165039</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>-0.004124858161063338</v>
+        <v>-0.004124624119425047</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
@@ -9187,7 +9187,7 @@
         </is>
       </c>
       <c r="D64" s="3" t="n">
-        <v>24.28103828430176</v>
+        <v>24.28104019165039</v>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
@@ -9195,10 +9195,10 @@
         </is>
       </c>
       <c r="F64" s="3" t="n">
-        <v>27.17429733276367</v>
+        <v>27.17430114746094</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>0.1191571387757528</v>
+        <v>0.1191572079686052</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
@@ -9223,7 +9223,7 @@
         </is>
       </c>
       <c r="D65" s="3" t="n">
-        <v>27.17429733276367</v>
+        <v>27.17430114746094</v>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
@@ -9234,7 +9234,7 @@
         <v>18.47107696533203</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>-0.3202739802562728</v>
+        <v>-0.3202740756754329</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
@@ -9267,10 +9267,10 @@
         </is>
       </c>
       <c r="F66" s="3" t="n">
-        <v>18.59556198120117</v>
+        <v>18.59556007385254</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>0.006739456291735557</v>
+        <v>0.006739353030370099</v>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
@@ -9295,7 +9295,7 @@
         </is>
       </c>
       <c r="D67" s="3" t="n">
-        <v>18.59556198120117</v>
+        <v>18.59556007385254</v>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
@@ -9303,10 +9303,10 @@
         </is>
       </c>
       <c r="F67" s="3" t="n">
-        <v>15.10013675689697</v>
+        <v>15.10013484954834</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>-0.1879709377881579</v>
+        <v>-0.1879709570683575</v>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
@@ -9331,7 +9331,7 @@
         </is>
       </c>
       <c r="D68" s="3" t="n">
-        <v>15.10013675689697</v>
+        <v>15.10013484954834</v>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
@@ -9339,10 +9339,10 @@
         </is>
       </c>
       <c r="F68" s="3" t="n">
-        <v>18.09246826171875</v>
+        <v>18.09247207641602</v>
       </c>
       <c r="G68" s="3" t="n">
-        <v>0.1981658545877099</v>
+        <v>0.1981662585587558</v>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
@@ -9367,7 +9367,7 @@
         </is>
       </c>
       <c r="D69" s="3" t="n">
-        <v>18.09246826171875</v>
+        <v>18.09247207641602</v>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
@@ -9375,10 +9375,10 @@
         </is>
       </c>
       <c r="F69" s="3" t="n">
-        <v>15.03538513183594</v>
+        <v>15.03538703918457</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>-0.1689699318887956</v>
+        <v>-0.1689700016846472</v>
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
@@ -9403,7 +9403,7 @@
         </is>
       </c>
       <c r="D70" s="3" t="n">
-        <v>15.03538513183594</v>
+        <v>15.03538703918457</v>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
@@ -9414,7 +9414,7 @@
         <v>12.09545421600342</v>
       </c>
       <c r="G70" s="3" t="n">
-        <v>-0.1955341276631157</v>
+        <v>-0.1955342297154857</v>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
@@ -9519,10 +9519,10 @@
         </is>
       </c>
       <c r="F73" s="3" t="n">
-        <v>14.5653018951416</v>
+        <v>14.56530094146729</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>-0.1364415308901092</v>
+        <v>-0.1364415874322625</v>
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
@@ -9547,7 +9547,7 @@
         </is>
       </c>
       <c r="D74" s="3" t="n">
-        <v>14.5653018951416</v>
+        <v>14.56530094146729</v>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
@@ -9555,10 +9555,10 @@
         </is>
       </c>
       <c r="F74" s="3" t="n">
-        <v>19.47190284729004</v>
+        <v>19.47189712524414</v>
       </c>
       <c r="G74" s="3" t="n">
-        <v>0.3368691557148624</v>
+        <v>0.3368688503927728</v>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
@@ -9583,7 +9583,7 @@
         </is>
       </c>
       <c r="D75" s="3" t="n">
-        <v>19.47190284729004</v>
+        <v>19.47189712524414</v>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
@@ -9591,10 +9591,10 @@
         </is>
       </c>
       <c r="F75" s="3" t="n">
-        <v>23.13863563537598</v>
+        <v>23.13863754272461</v>
       </c>
       <c r="G75" s="3" t="n">
-        <v>0.1883089093471031</v>
+        <v>0.1883093564995657</v>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
@@ -9619,7 +9619,7 @@
         </is>
       </c>
       <c r="D76" s="3" t="n">
-        <v>23.13863563537598</v>
+        <v>23.13863754272461</v>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
@@ -9627,10 +9627,10 @@
         </is>
       </c>
       <c r="F76" s="3" t="n">
-        <v>27.68914222717285</v>
+        <v>27.68914031982422</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>0.1966627014446669</v>
+        <v>0.1966625203708421</v>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
@@ -9655,7 +9655,7 @@
         </is>
       </c>
       <c r="D77" s="3" t="n">
-        <v>27.68914222717285</v>
+        <v>27.68914031982422</v>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
@@ -9663,10 +9663,10 @@
         </is>
       </c>
       <c r="F77" s="3" t="n">
-        <v>27.66123008728027</v>
+        <v>27.66123199462891</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>-0.001008053614069193</v>
+        <v>-0.001007915914793878</v>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
@@ -9691,7 +9691,7 @@
         </is>
       </c>
       <c r="D78" s="3" t="n">
-        <v>27.66123008728027</v>
+        <v>27.66123199462891</v>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
@@ -9699,10 +9699,10 @@
         </is>
       </c>
       <c r="F78" s="3" t="n">
-        <v>37.71432876586914</v>
+        <v>37.71433258056641</v>
       </c>
       <c r="G78" s="3" t="n">
-        <v>0.363436428780211</v>
+        <v>0.3634364726737245</v>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
@@ -9727,7 +9727,7 @@
         </is>
       </c>
       <c r="D79" s="3" t="n">
-        <v>37.71432876586914</v>
+        <v>37.71433258056641</v>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
@@ -9738,7 +9738,7 @@
         <v>42.17256546020508</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>0.1182106865009505</v>
+        <v>0.1182105733971262</v>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
@@ -9807,10 +9807,10 @@
         </is>
       </c>
       <c r="F81" s="3" t="n">
-        <v>49.20398330688477</v>
+        <v>49.20398712158203</v>
       </c>
       <c r="G81" s="3" t="n">
-        <v>0.05619655619364927</v>
+        <v>0.05619663807868869</v>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
@@ -9835,7 +9835,7 @@
         </is>
       </c>
       <c r="D82" s="3" t="n">
-        <v>49.20398330688477</v>
+        <v>49.20398712158203</v>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
@@ -9843,10 +9843,10 @@
         </is>
       </c>
       <c r="F82" s="3" t="n">
-        <v>43.36946868896484</v>
+        <v>43.36948013305664</v>
       </c>
       <c r="G82" s="3" t="n">
-        <v>-0.1185780952231065</v>
+        <v>-0.1185779309735295</v>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
@@ -9871,7 +9871,7 @@
         </is>
       </c>
       <c r="D83" s="3" t="n">
-        <v>43.36946868896484</v>
+        <v>43.36948013305664</v>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
@@ -9879,10 +9879,10 @@
         </is>
       </c>
       <c r="F83" s="3" t="n">
-        <v>40.65856170654297</v>
+        <v>40.6585693359375</v>
       </c>
       <c r="G83" s="3" t="n">
-        <v>-0.062507267540302</v>
+        <v>-0.06250733900434413</v>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
@@ -9907,7 +9907,7 @@
         </is>
       </c>
       <c r="D84" s="3" t="n">
-        <v>40.65856170654297</v>
+        <v>40.6585693359375</v>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
@@ -9915,10 +9915,10 @@
         </is>
       </c>
       <c r="F84" s="3" t="n">
-        <v>46.63073348999023</v>
+        <v>46.63072967529297</v>
       </c>
       <c r="G84" s="3" t="n">
-        <v>0.1468859579084962</v>
+        <v>0.1468856488778802</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -9943,7 +9943,7 @@
         </is>
       </c>
       <c r="D85" s="3" t="n">
-        <v>46.63073348999023</v>
+        <v>46.63072967529297</v>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
@@ -9951,10 +9951,10 @@
         </is>
       </c>
       <c r="F85" s="3" t="n">
-        <v>49.37887573242188</v>
+        <v>49.37887954711914</v>
       </c>
       <c r="G85" s="3" t="n">
-        <v>0.05893414142888309</v>
+        <v>0.05893430986310011</v>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
@@ -9979,7 +9979,7 @@
         </is>
       </c>
       <c r="D86" s="3" t="n">
-        <v>49.37887573242188</v>
+        <v>49.37887954711914</v>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
@@ -9987,10 +9987,10 @@
         </is>
       </c>
       <c r="F86" s="3" t="n">
-        <v>61.34918212890625</v>
+        <v>61.34918594360352</v>
       </c>
       <c r="G86" s="3" t="n">
-        <v>0.2424175564739466</v>
+        <v>0.2424175377463125</v>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
@@ -10015,7 +10015,7 @@
         </is>
       </c>
       <c r="D87" s="3" t="n">
-        <v>61.34918212890625</v>
+        <v>61.34918594360352</v>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
@@ -10023,10 +10023,10 @@
         </is>
       </c>
       <c r="F87" s="3" t="n">
-        <v>78.88337707519531</v>
+        <v>78.88336181640625</v>
       </c>
       <c r="G87" s="3" t="n">
-        <v>0.2858097587910202</v>
+        <v>0.2858094301189487</v>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
@@ -10051,7 +10051,7 @@
         </is>
       </c>
       <c r="D88" s="3" t="n">
-        <v>78.88337707519531</v>
+        <v>78.88336181640625</v>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
@@ -10062,7 +10062,7 @@
         <v>90.09909820556641</v>
       </c>
       <c r="G88" s="3" t="n">
-        <v>0.1421810468342366</v>
+        <v>0.1421812677718244</v>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
@@ -10131,10 +10131,10 @@
         </is>
       </c>
       <c r="F90" s="3" t="n">
-        <v>109.3212738037109</v>
+        <v>109.3212890625</v>
       </c>
       <c r="G90" s="3" t="n">
-        <v>0.2688708902152934</v>
+        <v>0.2688710673211081</v>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
@@ -10159,7 +10159,7 @@
         </is>
       </c>
       <c r="D91" s="3" t="n">
-        <v>109.3212738037109</v>
+        <v>109.3212890625</v>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
@@ -10167,10 +10167,10 @@
         </is>
       </c>
       <c r="F91" s="3" t="n">
-        <v>123.1988677978516</v>
+        <v>123.198860168457</v>
       </c>
       <c r="G91" s="3" t="n">
-        <v>0.1269432152707823</v>
+        <v>0.1269429881861628</v>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
@@ -10195,7 +10195,7 @@
         </is>
       </c>
       <c r="D92" s="3" t="n">
-        <v>123.1988677978516</v>
+        <v>123.198860168457</v>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
@@ -10203,10 +10203,10 @@
         </is>
       </c>
       <c r="F92" s="3" t="n">
-        <v>116.6968536376953</v>
+        <v>116.6968612670898</v>
       </c>
       <c r="G92" s="3" t="n">
-        <v>-0.05277657397651536</v>
+        <v>-0.05277645338988224</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -10231,7 +10231,7 @@
         </is>
       </c>
       <c r="D93" s="3" t="n">
-        <v>116.6968536376953</v>
+        <v>116.6968612670898</v>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
@@ -10242,7 +10242,7 @@
         <v>119.0403747558594</v>
       </c>
       <c r="G93" s="3" t="n">
-        <v>0.02008212771048568</v>
+        <v>0.02008206101966881</v>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
@@ -10275,10 +10275,10 @@
         </is>
       </c>
       <c r="F94" s="3" t="n">
-        <v>121.1150207519531</v>
+        <v>121.1150283813477</v>
       </c>
       <c r="G94" s="3" t="n">
-        <v>0.01742808690201669</v>
+        <v>0.0174281509928309</v>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
@@ -10303,7 +10303,7 @@
         </is>
       </c>
       <c r="D95" s="3" t="n">
-        <v>121.1150207519531</v>
+        <v>121.1150283813477</v>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
@@ -10311,10 +10311,10 @@
         </is>
       </c>
       <c r="F95" s="3" t="n">
-        <v>132.4047546386719</v>
+        <v>132.4047393798828</v>
       </c>
       <c r="G95" s="3" t="n">
-        <v>0.09321497710709581</v>
+        <v>0.09321478225631852</v>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
@@ -10339,7 +10339,7 @@
         </is>
       </c>
       <c r="D96" s="3" t="n">
-        <v>132.4047546386719</v>
+        <v>132.4047393798828</v>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
@@ -10350,7 +10350,7 @@
         <v>137.8800354003906</v>
       </c>
       <c r="G96" s="3" t="n">
-        <v>0.04135259928286272</v>
+        <v>0.04135271929200823</v>
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
@@ -10383,10 +10383,10 @@
         </is>
       </c>
       <c r="F97" s="3" t="n">
-        <v>133.9398498535156</v>
+        <v>133.9398651123047</v>
       </c>
       <c r="G97" s="3" t="n">
-        <v>-0.02857691133769347</v>
+        <v>-0.02857680067055435</v>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
@@ -10411,7 +10411,7 @@
         </is>
       </c>
       <c r="D98" s="3" t="n">
-        <v>133.9398498535156</v>
+        <v>133.9398651123047</v>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
@@ -10422,7 +10422,7 @@
         <v>119.7569351196289</v>
       </c>
       <c r="G98" s="3" t="n">
-        <v>-0.1058901794305278</v>
+        <v>-0.1058902812899192</v>
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
@@ -10455,10 +10455,10 @@
         </is>
       </c>
       <c r="F99" s="3" t="n">
-        <v>124.5942993164062</v>
+        <v>124.5942840576172</v>
       </c>
       <c r="G99" s="3" t="n">
-        <v>0.04039318634820721</v>
+        <v>0.04039305893354816</v>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
@@ -10483,7 +10483,7 @@
         </is>
       </c>
       <c r="D100" s="3" t="n">
-        <v>124.5942993164062</v>
+        <v>124.5942840576172</v>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
@@ -10491,10 +10491,10 @@
         </is>
       </c>
       <c r="F100" s="3" t="n">
-        <v>108.1073532104492</v>
+        <v>108.1073608398438</v>
       </c>
       <c r="G100" s="3" t="n">
-        <v>-0.1323250437332495</v>
+        <v>-0.1323248762370933</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -10519,7 +10519,7 @@
         </is>
       </c>
       <c r="D101" s="3" t="n">
-        <v>108.1073532104492</v>
+        <v>108.1073608398438</v>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
@@ -10530,7 +10530,7 @@
         <v>108.64599609375</v>
       </c>
       <c r="G101" s="3" t="n">
-        <v>0.004982481462220356</v>
+        <v>0.004982410538207693</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
@@ -10635,10 +10635,10 @@
         </is>
       </c>
       <c r="F104" s="3" t="n">
-        <v>177.4348602294922</v>
+        <v>177.4348754882812</v>
       </c>
       <c r="G104" s="3" t="n">
-        <v>0.1258305979143173</v>
+        <v>0.125830694731885</v>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
@@ -10663,7 +10663,7 @@
         </is>
       </c>
       <c r="D105" s="3" t="n">
-        <v>177.4348602294922</v>
+        <v>177.4348754882812</v>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
@@ -10671,10 +10671,10 @@
         </is>
       </c>
       <c r="F105" s="3" t="n">
-        <v>173.7538909912109</v>
+        <v>173.75390625</v>
       </c>
       <c r="G105" s="3" t="n">
-        <v>-0.0207454681313487</v>
+        <v>-0.02074546634730989</v>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
@@ -10699,7 +10699,7 @@
         </is>
       </c>
       <c r="D106" s="3" t="n">
-        <v>173.7538909912109</v>
+        <v>173.75390625</v>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
@@ -10710,7 +10710,7 @@
         <v>186.1340637207031</v>
       </c>
       <c r="G106" s="3" t="n">
-        <v>0.07125119707459349</v>
+        <v>0.07125110299903326</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -10779,10 +10779,10 @@
         </is>
       </c>
       <c r="F108" s="3" t="n">
-        <v>176.5769500732422</v>
+        <v>176.5769653320312</v>
       </c>
       <c r="G108" s="3" t="n">
-        <v>-0.1258827644807442</v>
+        <v>-0.1258826889444383</v>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
@@ -10807,7 +10807,7 @@
         </is>
       </c>
       <c r="D109" s="3" t="n">
-        <v>176.5769500732422</v>
+        <v>176.5769653320312</v>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
@@ -10818,7 +10818,7 @@
         <v>186.0646057128906</v>
       </c>
       <c r="G109" s="3" t="n">
-        <v>0.05373099736807707</v>
+        <v>0.05373090631056576</v>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
@@ -10887,10 +10887,10 @@
         </is>
       </c>
       <c r="F111" s="3" t="n">
-        <v>176.7763366699219</v>
+        <v>176.7763519287109</v>
       </c>
       <c r="G111" s="3" t="n">
-        <v>-0.07293472316669725</v>
+        <v>-0.07293464314527709</v>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
@@ -10915,7 +10915,7 @@
         </is>
       </c>
       <c r="D112" s="3" t="n">
-        <v>176.7763366699219</v>
+        <v>176.7763519287109</v>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
@@ -10923,10 +10923,10 @@
         </is>
       </c>
       <c r="F112" s="3" t="n">
-        <v>174.0022583007812</v>
+        <v>174.0022735595703</v>
       </c>
       <c r="G112" s="3" t="n">
-        <v>-0.0156925888464382</v>
+        <v>-0.01569258749190239</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -10951,7 +10951,7 @@
         </is>
       </c>
       <c r="D113" s="3" t="n">
-        <v>174.0022583007812</v>
+        <v>174.0022735595703</v>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
@@ -10959,10 +10959,10 @@
         </is>
       </c>
       <c r="F113" s="3" t="n">
-        <v>199.1148681640625</v>
+        <v>199.1148834228516</v>
       </c>
       <c r="G113" s="3" t="n">
-        <v>0.1443234709050238</v>
+        <v>0.1443234582488593</v>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
@@ -10987,7 +10987,7 @@
         </is>
       </c>
       <c r="D114" s="3" t="n">
-        <v>199.1148681640625</v>
+        <v>199.1148834228516</v>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
@@ -10998,7 +10998,7 @@
         <v>210.6584930419922</v>
       </c>
       <c r="G114" s="3" t="n">
-        <v>0.05797470065579535</v>
+        <v>0.05797461957992356</v>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
@@ -11570,7 +11570,7 @@
         <v>3.499741379310346</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>4.766270954987323</v>
+        <v>4.766271550373824</v>
       </c>
     </row>
     <row r="3">
@@ -11583,7 +11583,7 @@
         <v>3.42868537831944</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>3.894525960227657</v>
+        <v>3.894525878804123</v>
       </c>
     </row>
     <row r="4">
@@ -11622,7 +11622,7 @@
         <v>3.696486486486487</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>12.17800676700963</v>
+        <v>12.17801071817231</v>
       </c>
     </row>
     <row r="7">
@@ -11635,7 +11635,7 @@
         <v>-0.8680000000000002</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>-8.791782359687629</v>
+        <v>-8.791787902916088</v>
       </c>
     </row>
     <row r="8">
@@ -11648,7 +11648,7 @@
         <v>21.97</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>38.54459413790421</v>
+        <v>38.54458842745316</v>
       </c>
     </row>
     <row r="9">
@@ -11661,7 +11661,7 @@
         <v>-2.2</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>-32.02739802562728</v>
+        <v>-32.02740756754329</v>
       </c>
     </row>
     <row r="10">
@@ -11674,7 +11674,7 @@
         <v>3.499741379310346</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>4.766270954987323</v>
+        <v>4.766271550373824</v>
       </c>
     </row>
     <row r="11">
@@ -11687,7 +11687,7 @@
         <v>3.972276416934467</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>13.40454352252829</v>
+        <v>13.40454892611204</v>
       </c>
     </row>
     <row r="12">
@@ -11700,7 +11700,7 @@
         <v>2.651927277101982</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>-0.03153827838289425</v>
+        <v>-0.03153799374004402</v>
       </c>
     </row>
     <row r="13">
@@ -11713,7 +11713,7 @@
         <v>8.629009524988723</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.1667139613486102</v>
+        <v>0.1667112763682104</v>
       </c>
     </row>
     <row r="14">
@@ -11726,7 +11726,7 @@
         <v>0.8810417533861374</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.355571299162624</v>
+        <v>0.355571200243011</v>
       </c>
     </row>
     <row r="15">
@@ -11739,7 +11739,7 @@
         <v>14.56591488300176</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.6764342599160132</v>
+        <v>0.6764341416878362</v>
       </c>
     </row>
     <row r="16">
@@ -11752,7 +11752,7 @@
         <v>94.54147465437789</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>2.533825421920513</v>
+        <v>2.533824646442687</v>
       </c>
     </row>
   </sheetData>

</xml_diff>